<commit_message>
handling the canada , heux text
</commit_message>
<xml_diff>
--- a/yt_multi_language_ui_validator/src/main/resources/data/HypeLiveWords.xlsx
+++ b/yt_multi_language_ui_validator/src/main/resources/data/HypeLiveWords.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="132">
   <si>
     <t>Applied Language</t>
   </si>
@@ -405,6 +405,9 @@
   </si>
   <si>
     <t>라이브</t>
+  </si>
+  <si>
+    <t>Jeux vidéo</t>
   </si>
 </sst>
 </file>
@@ -452,9 +455,9 @@
   <dimension ref="A1:C54"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="20.20703125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="19.72265625" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="18.625" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" bestFit="true" customWidth="true" width="20.20703125"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" width="19.72265625"/>
+    <col min="3" max="3" bestFit="true" customWidth="true" width="18.625"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -652,7 +655,7 @@
         <v>36</v>
       </c>
       <c r="C18" t="s" s="0">
-        <v>37</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19">

</xml_diff>